<commit_message>
Update full 12-sheet Student Project Runbook with complete academic and technical data
</commit_message>
<xml_diff>
--- a/SIST_Student_FullStack_Project_Runbook.xlsx
+++ b/SIST_Student_FullStack_Project_Runbook.xlsx
@@ -632,11 +632,15 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Department of Computer Science and Engineering — Artificial Intelligence (CSE AI) | Capstone Runbook</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
+          <t>Department of Computer Science and Engineering — Artificial Intelligence (CSE AI)</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Capstone Runbook — TEAM-14</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -647,7 +651,7 @@
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Student 1 (Lead / Full Name):</t>
+          <t>Student 1 (Lead Architect):</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
@@ -669,12 +673,12 @@
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Student 2 (Partner Full Name):</t>
+          <t>Student 2 (Frontend Specialist):</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Alexiya fernando</t>
+          <t>Alexiya Fernando</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -696,7 +700,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>B.E. CSE (Artificial Intelligence) — 3rd Year</t>
+          <t>Computer Science and Engineering - AI (3rd Year)</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -706,7 +710,7 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>2024-2028/section [A5]</t>
+          <t>2024-2028 / Section A5 (Team ID: TEAM-14)</t>
         </is>
       </c>
     </row>
@@ -750,7 +754,7 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Placement Training Cell / Trainer</t>
+          <t>Placement Training Cell / SIST Academic Lead</t>
         </is>
       </c>
     </row>
@@ -762,7 +766,7 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Phase 1: Project Charter &amp; Requirements Kickoff</t>
+          <t>2026-09-01 (Phase 1: Project Charter Kickoff)</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
@@ -772,11 +776,10 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Phase 4: Final Viva, Live Demo &amp; Cloud Pitch</t>
-        </is>
-      </c>
-    </row>
-    <row r="11"/>
+          <t>2026-09-19 (Phase 4: Final Viva &amp; Live Demo)</t>
+        </is>
+      </c>
+    </row>
     <row r="12" ht="24" customHeight="1">
       <c r="A12" s="6" t="inlineStr">
         <is>
@@ -833,7 +836,6 @@
         </is>
       </c>
     </row>
-    <row r="20"/>
     <row r="21" ht="24" customHeight="1">
       <c r="A21" s="6" t="inlineStr">
         <is>
@@ -1030,11 +1032,10 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>🔌 PHASE 3: DEVELOP — FULL-STACK WIRING &amp; FETCH API INTEGRATION</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
+          <t>🔌 PHASE 3: DEVELOP — FULL-STACK WIRING, FETCH API &amp; CORS INTEGRATION</t>
+        </is>
+      </c>
+    </row>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
         <is>
@@ -1070,7 +1071,7 @@
       </c>
       <c r="C4" s="9" t="inlineStr">
         <is>
-          <t>Intercepts login form, dispatches POST /api/auth/login, persists user role (PATIENT, DOCTOR, ADMIN) in browser localStorage, and executes role-based route protection.</t>
+          <t>Intercepts login form submit, dispatches POST /api/auth/login, persists authenticated user session role (PATIENT, DOCTOR, ADMIN) in browser localStorage, and executes client-side route guard protection.</t>
         </is>
       </c>
       <c r="D4" s="9" t="inlineStr">
@@ -1092,7 +1093,7 @@
       </c>
       <c r="C5" s="9" t="inlineStr">
         <is>
-          <t>On date input change, triggers async fetch to calculate available slots against doctor working hours and existing bookings; renders clickable slot buttons dynamically.</t>
+          <t>On date input change, triggers async fetch to calculate available slots against doctor working hours and existing bookings; renders clickable slot buttons dynamically with instant state update.</t>
         </is>
       </c>
       <c r="D5" s="9" t="inlineStr">
@@ -1114,7 +1115,7 @@
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>Submits appointment JSON payload; if another user claimed the slot milliseconds earlier, captures HTTP 409 Conflict and alerts patient immediately without crashing the page.</t>
+          <t>Submits appointment JSON payload; if another user claimed the slot milliseconds earlier, captures HTTP 409 Conflict and alerts patient immediately without crashing or reloading page.</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
@@ -1158,7 +1159,7 @@
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>Periodically queries GET /api/queue/doctor/{id}/today every 5 seconds, updating waiting room consultation badges and token counters dynamically without page flicker.</t>
+          <t>Periodically queries GET /api/queue/doctor/{id}/today every 5 seconds, updating waiting room consultation badges and token counters dynamically without visual flicker.</t>
         </is>
       </c>
       <c r="D8" s="9" t="inlineStr">
@@ -1196,7 +1197,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
         <is>
@@ -1237,7 +1237,7 @@
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>CORS policy blocked API requests when accessing frontend on alternate local origin (e.g. port 5500).</t>
+          <t>CORS policy blocked API requests when accessing frontend on alternate local origin (e.g. port 5500 Live Server).</t>
         </is>
       </c>
       <c r="C4" s="9" t="inlineStr">
@@ -1247,12 +1247,12 @@
       </c>
       <c r="D4" s="9" t="inlineStr">
         <is>
-          <t>Spring Boot backend on port 8080 did not include Access-Control-Allow-Origin headers for frontend origins.</t>
+          <t>Spring Boot backend on port 8080 did not include Access-Control-Allow-Origin response headers for cross-origin frontend requests.</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
         <is>
-          <t>Added @CrossOrigin(origins = "*") on all @RestController classes and served static frontend directly from src/main/resources/static.</t>
+          <t>Added @CrossOrigin(origins = "*") on all @RestController classes and configured static resources in Spring Boot.</t>
         </is>
       </c>
       <c r="F4" s="17" t="inlineStr">
@@ -1269,7 +1269,7 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>Race condition: simultaneous booking requests for the exact same doctor and slot created duplicate appointments.</t>
+          <t>Race condition: simultaneous booking requests for the exact same doctor, date, and slot created duplicate appointments.</t>
         </is>
       </c>
       <c r="C5" s="9" t="inlineStr">
@@ -1284,7 +1284,7 @@
       </c>
       <c r="E5" s="9" t="inlineStr">
         <is>
-          <t>Added database-level unique constraint on (doctor_id, appointment_date, slot_time) and custom SlotAlreadyBookedException mapped to HTTP 409 Conflict.</t>
+          <t>Added database-level composite unique constraint on (doctor_id, appointment_date, appointment_time) and custom SlotAlreadyBookedException mapped to HTTP 409 Conflict.</t>
         </is>
       </c>
       <c r="F5" s="17" t="inlineStr">
@@ -1311,7 +1311,7 @@
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>Bidirectional JPA @OneToMany and @ManyToOne references caused Jackson JSON serializer to loop indefinitely.</t>
+          <t>Bidirectional JPA @OneToMany and @ManyToOne references caused Jackson JSON serializer to loop indefinitely between parent and child objects.</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -1380,11 +1380,10 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>🚀 PHASE 4: DEPLOY — CLOUD DEPLOYMENT &amp; 3-MINUTE PITCH SCRIPT</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
+          <t>🚀 PHASE 4: DEPLOY — CLOUD DEPLOYMENT &amp; 3-MINUTE VIVA PITCH SCRIPT</t>
+        </is>
+      </c>
+    </row>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
         <is>
@@ -1420,12 +1419,12 @@
       </c>
       <c r="C4" s="9" t="inlineStr">
         <is>
-          <t>https://github.com/clinic-appointment-booking-system/clinic-appointment-booking-system</t>
+          <t>https://github.com/Diwakar24281/clinic-appointment-system</t>
         </is>
       </c>
       <c r="D4" s="15" t="inlineStr">
         <is>
-          <t>Verified Active</t>
+          <t>Verified Active &amp; Public</t>
         </is>
       </c>
     </row>
@@ -1437,7 +1436,7 @@
       </c>
       <c r="B5" s="10" t="inlineStr">
         <is>
-          <t>GitHub Pages / Vercel / Netlify</t>
+          <t>Embedded Tomcat / GitHub Pages / Port 8080</t>
         </is>
       </c>
       <c r="C5" s="9" t="inlineStr">
@@ -1447,7 +1446,7 @@
       </c>
       <c r="D5" s="15" t="inlineStr">
         <is>
-          <t>Live in Browser</t>
+          <t>Live &amp; Responsive</t>
         </is>
       </c>
     </row>
@@ -1459,17 +1458,17 @@
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
-          <t>Render.com / Railway / Cloud VM</t>
+          <t>Spring Boot 3.2.5 REST Server</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>http://localhost:8080/api/appointments (Spring Boot 3.2.5 REST Server on Port 8080)</t>
+          <t>http://localhost:8080/api/appointments (Port 8080 RESTful API)</t>
         </is>
       </c>
       <c r="D6" s="15" t="inlineStr">
         <is>
-          <t>Responding 200 OK</t>
+          <t>Responding 200 OK / 201 Created</t>
         </is>
       </c>
     </row>
@@ -1495,24 +1494,24 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
-    <row r="9"/>
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>🎤 3-MINUTE TECHNICAL VIVA PITCH SCRIPT FOR RECRUITERS</t>
+          <t>🎤 3-MINUTE TECHNICAL VIVA PITCH SCRIPT (DIVIDED ACROSS TEAM-14 MEMBERS)</t>
         </is>
       </c>
     </row>
     <row r="11" ht="45" customHeight="1">
       <c r="A11" s="18" t="inlineStr">
         <is>
-          <t>Minute 1: The Problem &amp; Value</t>
+          <t>Minute 1: Problem &amp; System Scope (Lead Architect - N.Diwakar)</t>
         </is>
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>Hello! We built Clinic Appointment Booking System — an end-to-end Clinic Appointment Booking and Real-Time Queue Management System. Traditional outpatient clinics suffer from chaotic walk-ins, excessive waiting times (often 2+ hours), frequent double-booking conflicts, and fragile paper prescriptions. Clinic Appointment Booking System provides an automated 3-tier full-stack solution featuring 30-minute slot reservation, strict double-booking prevention, automated daily token generation, a live public waiting room board, and structured digital prescriptions.</t>
+          <t>Good morning respected evaluators! We are TEAM-14, presenting the Clinic Appointment Booking and Queue Management System.
+Traditional outpatient clinics face severe operational bottlenecks: chaotic walk-in lines, patient wait times exceeding 2 hours, frequent double-booking scheduling collisions, lack of live queue visibility for waiting patients, and fragile paper prescriptions prone to damage and loss.
+To solve this, our full-stack solution delivers automated 30-minute slot reservation, strict database-level double-booking prevention, automated doctor-isolated daily token generation (Token #1, #2...), a live 5-second public waiting room display board, and structured digital multi-medicine prescriptions.</t>
         </is>
       </c>
       <c r="C11" s="19" t="n"/>
@@ -1521,12 +1520,15 @@
     <row r="12" ht="45" customHeight="1">
       <c r="A12" s="18" t="inlineStr">
         <is>
-          <t>Minute 2: System Architecture &amp; Tech Stack</t>
+          <t>Minute 2: 3-Tier Architecture &amp; Tech Stack (Lead Architect - N.Diwakar &amp; Frontend Specialist - Alexiya Fernando)</t>
         </is>
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>Architecturally, Clinic Appointment Booking System is engineered across 3 decoupled layers: Tier 1 is a semantic HTML5, CSS3 Grid, and Vanilla JavaScript (ES6+) Fetch API client with dedicated portals for Patients, Doctors, Admins, and Public Waiting displays. Tier 2 is a Java 17 Spring Boot 3.2.5 RESTful backend implementing a layered architecture: Controllers handling HTTP contracts, a Service layer enforcing business rules and concurrency locks, and Spring Data JPA repositories with Hibernate ORM. Tier 3 is a MySQL 8.0 relational database in 3NF with composite unique constraints and ACID compliance.</t>
+          <t>Architecturally, our system is engineered across 3 robust, decoupled tiers:
+• Tier 1 (Frontend): Developed using semantic HTML5, CSS3 Grid/Flexbox design tokens, and modular Vanilla JavaScript (ES6+) Fetch API interfacing seamlessly across Patient, Doctor, Admin, and Public Waiting Room portals.
+• Tier 2 (Backend Engine): Java 17 Spring Boot 3.2.5 REST backend with a strict 3-layer architecture: Controllers managing HTTP contracts, Service layer enforcing business validation and concurrency locks, and Spring Data JPA repositories.
+• Tier 3 (Database): MySQL 8.0 normalized in 3NF with composite unique constraints (uk_doctor_slot) and HikariCP connection pooling, ensuring strict ACID transactions and sub-200ms latency.</t>
         </is>
       </c>
       <c r="C12" s="19" t="n"/>
@@ -1535,12 +1537,16 @@
     <row r="13" ht="45" customHeight="1">
       <c r="A13" s="18" t="inlineStr">
         <is>
-          <t>Minute 3: Live Demo &amp; Engineering Robustness</t>
+          <t>Minute 3: Live Demonstration &amp; Robustness (Frontend Specialist - Alexiya Fernando)</t>
         </is>
       </c>
       <c r="B13" s="9" t="inlineStr">
         <is>
-          <t>In our live demo: First, a patient selects Dr. Ramesh Kumar, picks an available 10:00 AM slot, and receives instant Token #1. If another patient attempts to book the exact same slot, the system immediately rejects it with HTTP 409 Conflict. Next, in the Doctor Dashboard, the doctor clicks "Call Next Patient", updating the consultation status in real time and reflecting immediately on the live waiting room display board. Finally, the doctor creates a digital prescription with multi-row medications, which marks the visit COMPLETED and allows the patient to view and print their digital prescription instantly. We resolved CORS, circular serialization, and concurrency edge cases with systematic engineering.</t>
+          <t>During our live demonstration:
+1. Patient Portal: A patient selects Dr. Ramesh Kumar, chooses a 10:00 AM slot, and receives instant Token #1. When another user attempts to book the identical slot, the system immediately rejects it with HTTP 409 Conflict.
+2. Doctor Dashboard: The doctor clicks 'Call Next Patient', transitioning the token status to IN_CONSULTATION, which immediately reflects on the live waiting room display board via 5-second asynchronous polling.
+3. Digital Prescription: The doctor enters diagnosis, clinical notes, and multi-row medication items, clicking 'Save' to transition the visit to COMPLETED and generate a printable digital prescription invoice.
+We resolved CORS, Jackson circular serialization, and race condition challenges to build a production-grade system ready for deployment.</t>
         </is>
       </c>
       <c r="C13" s="19" t="n"/>
@@ -1563,7 +1569,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="56" customWidth="1" min="1" max="1"/>
@@ -1574,11 +1580,10 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>📋 PHASE 1: DEFINE — PROBLEM STATEMENT &amp; PROJECT SCOPE</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
+          <t>📋 PHASE 1: DEFINE — PROBLEM STATEMENT, MOSCOW TIERS &amp; NFRS</t>
+        </is>
+      </c>
+    </row>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
         <is>
@@ -1592,7 +1597,7 @@
       </c>
       <c r="C3" s="13" t="inlineStr">
         <is>
-          <t>Student Team Project Response (Edit &amp; Complete)</t>
+          <t>Student Team Project Response (TEAM-14: Clinic Appointment Booking System)</t>
         </is>
       </c>
     </row>
@@ -1626,7 +1631,7 @@
       </c>
       <c r="C5" s="9" t="inlineStr">
         <is>
-          <t>Traditional outpatient clinics suffer from severe operational bottlenecks: chaotic walk-in lines, prolonged patient waiting times (often exceeding 2+ hours), frequent double-booking scheduling conflicts, lack of live queue visibility for waiting patients, and vulnerable paper-based prescriptions prone to illegibility, physical damage, and loss. This causes high patient dissatisfaction, doctor scheduling inefficiencies, and administrative burnout.</t>
+          <t>Traditional outpatient clinics suffer from chaotic walk-ins, excessive waiting times (often 2+ hours), frequent double-booking scheduling conflicts, lack of live queue visibility for waiting patients, and vulnerable paper-based prescriptions prone to illegibility, physical damage, and loss. This causes high patient dissatisfaction, doctor scheduling inefficiencies, and administrative burnout.</t>
         </is>
       </c>
     </row>
@@ -1672,32 +1677,72 @@
     <row r="8" ht="50" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>5. Core Value Metric (KPI)</t>
+          <t>5. MoSCoW Prioritization</t>
         </is>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>How will you quantify the technical success of this application?</t>
+          <t>Categorize project features into the 4 MoSCoW prioritization tiers.</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>100% elimination of double-booking collisions, 60% reduction in patient clinic waiting time via real-time queue tracking, sub-200ms REST API response latency, and 100% digital retention of clinical prescriptions.</t>
+          <t>• MUST HAVE (P0): Patient registration &amp; BCrypt login; Doctor directory with 30-min slot picker; Concurrency-safe appointment booking (409 Conflict check); Doctor daily queue &amp; 'Call Next Patient'; Electronic multi-row prescription generator; Live 5s waiting room display board.
+• SHOULD HAVE (P1): Admin doctor scheduling (Mon-Sat 9AM-1PM); Specialization management; Printable PDF-style prescription invoice; Appointment cancellation.
+• COULD HAVE (P2): Email/SMS notification alerts; Patient appointment history filtering; Doctor fee revenue analytics.
+• WON'T HAVE (P3 - Out of Scope): Commercial paid payment gateway integration; Telemedicine video streaming; Multi-hospital cross-tenant federation.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="50" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>6. Scope Exclusions (Out of Scope)</t>
+          <t>6. Non-Functional Requirements (NFRs)</t>
         </is>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
+          <t>Specify the 4 key engineering NFRs with quantifiable metrics.</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>1. Performance &amp; Latency: REST API response time &lt; 200ms for slot queries and appointment creations under 100 concurrent requests.
+2. Concurrency &amp; Data Integrity: 100% elimination of double-booking collisions via database-level unique constraint uk_doctor_slot (doctor_id, appointment_date, appointment_time) and pessimistic transaction locking.
+3. Security &amp; Compliance: BCrypt password hashing (strength 10), role-based route authentication (PATIENT, DOCTOR, ADMIN), and sanitized input DTO validation preventing SQL injection and XSS.
+4. Availability &amp; Reliability: Live waiting room poller resilient against transient network drops with automatic 5-second backoff recovery; zero data loss with MySQL InnoDB transactional engine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>7. Core Value Metric (KPI)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>How will you quantify the technical success of this application?</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>100% elimination of double-booking collisions, 60% reduction in patient clinic waiting time via real-time queue tracking, sub-200ms REST API response latency, and 100% digital retention of clinical prescriptions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>8. Scope Exclusions (Out of Scope)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
           <t>What complex features are intentionally deferred from this MVP?</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>Third-party commercial SMS/WhatsApp paid hardware gateways, live payment gateway escrow processing, and multi-hospital SaaS federation are scheduled for post-MVP production iterations.</t>
         </is>
@@ -1728,11 +1773,10 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>📝 PHASE 1: DEFINE — USER STORIES &amp; ACCEPTANCE CRITERIA</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
+          <t>📝 PHASE 1: DEFINE — USER STORIES &amp; GIVEN/WHEN/THEN ACCEPTANCE CRITERIA</t>
+        </is>
+      </c>
+    </row>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
         <is>
@@ -1788,10 +1832,8 @@
       </c>
       <c r="E4" s="9" t="inlineStr">
         <is>
-          <t>1. Fetches real-time 30-min time slots dynamically based on doctor weekly schedule.
-2. Prevents booking already reserved slots with HTTP 409 Conflict.
-3. Automatically generates sequential token number (e.g. Token #1, #2) for that doctor/date.
-4. Returns HTTP 201 Created with appointment confirmation details.</t>
+          <t>Criterion 1: Given a registered patient selects a doctor and future date, When they choose an available 30-minute time slot and confirm, Then the system creates an appointment, assigns a sequential token (e.g. Token #1), and returns HTTP 201 Created.
+Criterion 2: Given two patients simultaneously select the exact same doctor, date, and 10:00 AM slot, When both submit booking requests, Then the first request succeeds (201 Created) and the second request is immediately rejected with HTTP 409 Conflict.</t>
         </is>
       </c>
       <c r="F4" s="15" t="inlineStr">
@@ -1823,9 +1865,8 @@
       </c>
       <c r="E5" s="9" t="inlineStr">
         <is>
-          <t>1. Renders doctor cards in responsive CSS Grid with qualification, experience, fee, and timing.
-2. Client-side instant search filter by doctor name and specialization dropdown without page reload.
-3. Provides 1-click "Book Appointment" action directly on doctor card.</t>
+          <t>Criterion 1: Given a patient navigates to the Doctors directory, When the page loads, Then all active doctors are rendered in responsive cards showing name, specialization, qualification, experience, fee, and weekly schedule.
+Criterion 2: Given the doctor list is displayed, When the patient types a doctor's name or filters by specialization dropdown, Then the doctor list filters instantly in real-time without page reload.</t>
         </is>
       </c>
       <c r="F5" s="15" t="inlineStr">
@@ -1857,9 +1898,8 @@
       </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
-          <t>1. Displays real-time chronological queue of today's booked patients sorted by token number.
-2. 1-click "Call Next Patient" transitions appointment state to IN_CONSULTATION.
-3. Synchronously reflects across doctor dashboard and public waiting room display board.</t>
+          <t>Criterion 1: Given a logged-in doctor opens the Doctor Dashboard, When the page renders, Then today's patient queue is displayed in chronological order sorted by sequential token number with statuses (BOOKED, IN_CONSULTATION, COMPLETED).
+Criterion 2: Given waiting patients exist in the queue, When the doctor clicks 'Call Next Patient', Then the selected patient's status transitions to IN_CONSULTATION and updates synchronously across the dashboard and public waiting room display.</t>
         </is>
       </c>
       <c r="F6" s="15" t="inlineStr">
@@ -1891,9 +1931,8 @@
       </c>
       <c r="E7" s="9" t="inlineStr">
         <is>
-          <t>1. Captures diagnosis, clinical notes, follow-up date, and dynamic multi-row medicines (name, dosage, frequency, duration, instructions).
-2. Saves prescription entity, links to appointment, and transitions status to COMPLETED.
-3. Renders printable digital prescription view accessible by patient and doctor.</t>
+          <t>Criterion 1: Given a doctor is in consultation with an active patient, When the doctor enters diagnosis, clinical notes, and adds multiple medicine items (name, dosage, frequency, duration, instructions), Then clicking 'Save Prescription' persists the record and updates the appointment status to COMPLETED.
+Criterion 2: Given a completed appointment, When the patient or doctor opens the digital prescription page, Then a clean, printable PDF-style medical prescription document is rendered with all medication details.</t>
         </is>
       </c>
       <c r="F7" s="15" t="inlineStr">
@@ -1925,9 +1964,8 @@
       </c>
       <c r="E8" s="9" t="inlineStr">
         <is>
-          <t>1. Real-time high-visibility display showing "Current in Consultation", "Next in Line", and "Waiting Count".
-2. Automated periodic polling every 5 seconds using JavaScript Fetch API without page reload.
-3. Clean, high-contrast responsive display suitable for clinic TV monitors.</t>
+          <t>Criterion 1: Given the public waiting room display board is open on a clinic monitor, When doctor consultation statuses change, Then the display updates 'Current in Consultation', 'Next in Line', and 'Total Waiting' within 5 seconds via background polling without page refresh.
+Criterion 2: Given no patients are currently in consultation, When the queue is fetched, Then the board gracefully displays 'No patient currently in consultation' and shows the upcoming scheduled tokens.</t>
         </is>
       </c>
       <c r="F8" s="15" t="inlineStr">
@@ -1959,9 +1997,8 @@
       </c>
       <c r="E9" s="9" t="inlineStr">
         <is>
-          <t>1. Add/edit doctors with specialization, qualifications, experience, and consultation fees.
-2. Configure weekly availability slots (e.g. MONDAY to SATURDAY 09:00 - 13:00).
-3. View clinic KPI statistics (total doctors, active patients, appointments today).</t>
+          <t>Criterion 1: Given an authenticated administrator, When they create a new doctor with user credentials, specialization, fee, and weekly schedule (e.g. Mon-Sat 09:00-13:00), Then the new doctor is persisted in MySQL and becomes immediately available in patient slot booking.
+Criterion 2: Given the admin dashboard is loaded, When stats are requested, Then aggregate KPI cards display total doctors, registered patients, today's total appointments, and completed visits accurately.</t>
         </is>
       </c>
       <c r="F9" s="15" t="inlineStr">
@@ -1981,7 +2018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="61" customWidth="1" min="1" max="1"/>
@@ -1992,11 +2029,10 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>📐 PHASE 2: DESIGN — SYSTEM ARCHITECTURE &amp; DRAW.IO MODELING</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
+          <t>📐 PHASE 2: DESIGN — SYSTEM ARCHITECTURE, PORTS &amp; DRAW.IO SPECIFICATIONS</t>
+        </is>
+      </c>
+    </row>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
         <is>
@@ -2027,7 +2063,7 @@
       </c>
       <c r="C4" s="9" t="inlineStr">
         <is>
-          <t>Tool: Draw.io Web App (https://app.diagrams.net - Export as PNG/SVG/XML)</t>
+          <t>Tool: Draw.io Web App (https://app.diagrams.net - Exported as PNG/SVG in project repository presentation/ directory)</t>
         </is>
       </c>
     </row>
@@ -2040,12 +2076,12 @@
       <c r="B5" s="14" t="inlineStr">
         <is>
           <t>Draw a 'Browser' container representing the Client Frontend.
-Specify: Origin Port 5500, HTML5 UI, CSS Grid Layout, Vanilla JS Fetch API.</t>
+Specify: Origin Port 5500 / 8080, HTML5 UI, CSS Grid Layout, Vanilla JS Fetch API.</t>
         </is>
       </c>
       <c r="C5" s="9" t="inlineStr">
         <is>
-          <t>Tier 1: Client Web Application (HTML5, CSS3 Grid/Flexbox, Vanilla JS ES6+, Fetch API, Port 8080/Static - Patient, Doctor, Admin &amp; Waiting Room Portals)</t>
+          <t>Tier 1: Client Web Application (HTML5, CSS3 Grid/Flexbox, Vanilla JS ES6+, Fetch API, Port 8080/Static &amp; Port 5500 Dev Server - Patient Portal, Doctor Console, Admin Dashboard &amp; Public Waiting Room Display)</t>
         </is>
       </c>
     </row>
@@ -2063,7 +2099,7 @@
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>Protocol: HTTP/1.1 REST API (JSON payloads, @CrossOrigin, HTTP Status Codes 200 OK, 201 Created, 400 Bad Request, 404 Not Found, 409 Conflict)</t>
+          <t>Protocol: HTTP/1.1 REST API over Port 8080 (JSON payloads, @CrossOrigin enabled, Standard HTTP Status Codes: 200 OK, 201 Created, 400 Bad Request, 404 Not Found, 409 Conflict)</t>
         </is>
       </c>
     </row>
@@ -2081,7 +2117,7 @@
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
-          <t>Tier 2: Spring Boot 3.2.5 REST Backend (Controllers -&gt; Service Layer with Business Validation &amp; Concurrency Locks -&gt; Spring Data JPA Repositories -&gt; Hibernate ORM)</t>
+          <t>Tier 2: Spring Boot 3.2.5 REST Engine (Port 8080: Embedded Tomcat, REST Controllers -&gt; Service Layer with 30-min Slot Validation &amp; Concurrency Double-Booking Lock -&gt; Spring Data JPA Repositories -&gt; Hibernate ORM)</t>
         </is>
       </c>
     </row>
@@ -2099,7 +2135,7 @@
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>Driver: MySQL Connector/J with HikariCP Connection Pool over TCP/IP (Port 3306)</t>
+          <t>Driver: MySQL Connector/J with HikariCP Connection Pool over TCP/IP (Port 3306, serverTimezone=UTC, allowPublicKeyRetrieval=true)</t>
         </is>
       </c>
     </row>
@@ -2112,29 +2148,51 @@
       <c r="B9" s="14" t="inlineStr">
         <is>
           <t>Draw a 'Database Cylinder' shape representing MySQL 8.0 on disk.
-Label: Target schema and tables (e.g. app_db.orders, app_db.users).</t>
+Label: Target schema and tables (clinic_db schema).</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>Tier 3: MySQL 8.0 Relational Database (clinic_db schema: users, specializations, doctors, doctor_availabilities, patients, appointments, prescriptions, prescription_medicines)</t>
+          <t>Tier 3: MySQL 8.0 Relational Database (Port 3306: clinic_db schema with 8 normalized 3NF tables: users, specializations, doctors, doctor_availability, patients, appointments, prescriptions, prescription_medicines with composite unique constraints)</t>
         </is>
       </c>
     </row>
     <row r="10" ht="40" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Step 7: Diagram Embed / Link</t>
+          <t>Step 7: Data Flow &amp; Concurrency Pipeline</t>
         </is>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
+          <t>Detail end-to-end data flow for appointment booking and queue polling.</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>1. Client dispatches Fetch API POST /api/appointments JSON payload to Port 8080.
+2. AppointmentController routes to AppointmentService within @Transactional boundary.
+3. Service performs slot overlap check and queries AppointmentRepository.findMaxTokenNumberByDoctorAndDate.
+4. Hibernate issues INSERT into appointments with uk_doctor_slot constraint.
+5. MySQL commits transaction; Spring Boot returns HTTP 201 with generated Token #.
+6. Waiting Room poller on Port 8080 triggers GET /api/queue/doctor/{id}/today every 5000ms to update live queue DOM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Step 8: Diagram Embed / Repository Link</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
           <t>Export your Draw.io diagram as high-resolution PNG or shareable link and paste here:</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr">
-        <is>
-          <t>Clinic Appointment Booking System 3-tier System Architecture diagram modeled on Draw.io illustrating presentation layer, Spring Boot business controllers/services/repositories, and MySQL relational database with ACID constraints.</t>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Draw.io Architecture Diagram saved in repository at presentation/clinic_appointment_system_presentation.pdf and presentation/presentation.html illustrating decoupled 3-tier layout across Port 5500/8080 -&gt; Port 8080 -&gt; Port 3306.</t>
         </is>
       </c>
     </row>
@@ -2163,11 +2221,10 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>🗄️ PHASE 2: DESIGN — MYSQL RELATIONAL DATABASE SCHEMA (3NF)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
+          <t>🗄️ PHASE 2: DESIGN — MYSQL RELATIONAL DATABASE SCHEMA (3NF DATA DICTIONARY)</t>
+        </is>
+      </c>
+    </row>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
         <is>
@@ -2240,7 +2297,7 @@
       </c>
       <c r="B5" s="10" t="inlineStr">
         <is>
-          <t>email</t>
+          <t>name</t>
         </is>
       </c>
       <c r="C5" s="9" t="inlineStr">
@@ -2250,7 +2307,7 @@
       </c>
       <c r="D5" s="15" t="inlineStr">
         <is>
-          <t>UNIQUE</t>
+          <t>NONE</t>
         </is>
       </c>
       <c r="E5" s="9" t="inlineStr">
@@ -2260,7 +2317,7 @@
       </c>
       <c r="F5" s="9" t="inlineStr">
         <is>
-          <t>User login email address with unique constraint</t>
+          <t>Full legal name of the user (Patient, Doctor, or Admin)</t>
         </is>
       </c>
     </row>
@@ -2272,17 +2329,17 @@
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
-          <t>password</t>
+          <t>email</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>VARCHAR(255)</t>
+          <t>VARCHAR(100)</t>
         </is>
       </c>
       <c r="D6" s="15" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>UNIQUE (uk_user_email)</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -2292,7 +2349,7 @@
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t>BCrypt hashed secure password string</t>
+          <t>Unique user email address used as login username credential</t>
         </is>
       </c>
     </row>
@@ -2304,12 +2361,12 @@
       </c>
       <c r="B7" s="10" t="inlineStr">
         <is>
-          <t>full_name</t>
+          <t>password</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
-          <t>VARCHAR(100)</t>
+          <t>VARCHAR(255)</t>
         </is>
       </c>
       <c r="D7" s="15" t="inlineStr">
@@ -2324,7 +2381,7 @@
       </c>
       <c r="F7" s="9" t="inlineStr">
         <is>
-          <t>Full legal name of the user</t>
+          <t>BCrypt hashed secure password string (cost factor 10)</t>
         </is>
       </c>
     </row>
@@ -2341,7 +2398,7 @@
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>VARCHAR(20)</t>
+          <t>ENUM('PATIENT', 'DOCTOR', 'ADMIN')</t>
         </is>
       </c>
       <c r="D8" s="15" t="inlineStr">
@@ -2356,7 +2413,7 @@
       </c>
       <c r="F8" s="9" t="inlineStr">
         <is>
-          <t>User role enum: PATIENT, DOCTOR, ADMIN</t>
+          <t>User authorization role discriminator enum</t>
         </is>
       </c>
     </row>
@@ -2368,12 +2425,12 @@
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t>phone_number</t>
+          <t>created_at</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>VARCHAR(20)</t>
+          <t>TIMESTAMP</t>
         </is>
       </c>
       <c r="D9" s="15" t="inlineStr">
@@ -2383,44 +2440,44 @@
       </c>
       <c r="E9" s="9" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>DEFAULT CURRENT_TIMESTAMP</t>
         </is>
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
-          <t>Contact phone number for notifications</t>
+          <t>User account registration timestamp</t>
         </is>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="10" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>specializations</t>
         </is>
       </c>
       <c r="B10" s="10" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>id</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>TIMESTAMP</t>
+          <t>BIGINT AUTO_INCREMENT</t>
         </is>
       </c>
       <c r="D10" s="15" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>PRIMARY KEY</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
         <is>
-          <t>DEFAULT CURRENT_TIMESTAMP</t>
+          <t>NOT NULL</t>
         </is>
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
-          <t>User account creation timestamp</t>
+          <t>Unique specialization primary key identifier</t>
         </is>
       </c>
     </row>
@@ -2432,17 +2489,17 @@
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>name</t>
         </is>
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>BIGINT AUTO_INCREMENT</t>
+          <t>VARCHAR(100)</t>
         </is>
       </c>
       <c r="D11" s="15" t="inlineStr">
         <is>
-          <t>PRIMARY KEY</t>
+          <t>UNIQUE (uk_spec_name)</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
@@ -2452,7 +2509,7 @@
       </c>
       <c r="F11" s="9" t="inlineStr">
         <is>
-          <t>Unique specialization primary key identifier</t>
+          <t>Medical specialization department title (e.g. Cardiology, Pediatrics)</t>
         </is>
       </c>
     </row>
@@ -2464,59 +2521,59 @@
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>description</t>
         </is>
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>VARCHAR(100)</t>
+          <t>VARCHAR(255)</t>
         </is>
       </c>
       <c r="D12" s="15" t="inlineStr">
         <is>
-          <t>UNIQUE</t>
+          <t>NONE</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
         <is>
-          <t>NOT NULL</t>
+          <t>NULL</t>
         </is>
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
-          <t>Medical specialization title (e.g. Cardiology, Pediatrics)</t>
+          <t>Detailed clinical scope description of the medical department</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="10" t="inlineStr">
         <is>
-          <t>specializations</t>
+          <t>doctors</t>
         </is>
       </c>
       <c r="B13" s="10" t="inlineStr">
         <is>
-          <t>description</t>
+          <t>id</t>
         </is>
       </c>
       <c r="C13" s="9" t="inlineStr">
         <is>
-          <t>TEXT</t>
+          <t>BIGINT AUTO_INCREMENT</t>
         </is>
       </c>
       <c r="D13" s="15" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>PRIMARY KEY</t>
         </is>
       </c>
       <c r="E13" s="9" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>NOT NULL</t>
         </is>
       </c>
       <c r="F13" s="9" t="inlineStr">
         <is>
-          <t>Detailed description of medical field and clinical scope</t>
+          <t>Unique doctor entity primary key identifier</t>
         </is>
       </c>
     </row>
@@ -2528,17 +2585,17 @@
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>user_id</t>
         </is>
       </c>
       <c r="C14" s="9" t="inlineStr">
         <is>
-          <t>BIGINT AUTO_INCREMENT</t>
+          <t>BIGINT</t>
         </is>
       </c>
       <c r="D14" s="15" t="inlineStr">
         <is>
-          <t>PRIMARY KEY</t>
+          <t>FOREIGN KEY &amp; UNIQUE</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2548,7 +2605,7 @@
       </c>
       <c r="F14" s="9" t="inlineStr">
         <is>
-          <t>Unique doctor primary key identifier</t>
+          <t>1:1 reference to users(id) ON DELETE CASCADE</t>
         </is>
       </c>
     </row>
@@ -2560,7 +2617,7 @@
       </c>
       <c r="B15" s="10" t="inlineStr">
         <is>
-          <t>user_id</t>
+          <t>specialization_id</t>
         </is>
       </c>
       <c r="C15" s="9" t="inlineStr">
@@ -2580,7 +2637,7 @@
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
-          <t>References users(id) ON DELETE CASCADE</t>
+          <t>Many:1 reference to specializations(id)</t>
         </is>
       </c>
     </row>
@@ -2592,27 +2649,27 @@
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>specialization_id</t>
+          <t>consultation_fee</t>
         </is>
       </c>
       <c r="C16" s="9" t="inlineStr">
         <is>
-          <t>BIGINT</t>
+          <t>DECIMAL(10,2)</t>
         </is>
       </c>
       <c r="D16" s="15" t="inlineStr">
         <is>
-          <t>FOREIGN KEY</t>
+          <t>NONE</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
         <is>
-          <t>NOT NULL</t>
+          <t>NOT NULL DEFAULT 0.00</t>
         </is>
       </c>
       <c r="F16" s="9" t="inlineStr">
         <is>
-          <t>References specializations(id)</t>
+          <t>Outpatient doctor consultation fee amount in INR</t>
         </is>
       </c>
     </row>
@@ -2624,12 +2681,12 @@
       </c>
       <c r="B17" s="10" t="inlineStr">
         <is>
-          <t>qualification</t>
+          <t>is_available</t>
         </is>
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>VARCHAR(150)</t>
+          <t>BOOLEAN</t>
         </is>
       </c>
       <c r="D17" s="15" t="inlineStr">
@@ -2639,66 +2696,66 @@
       </c>
       <c r="E17" s="9" t="inlineStr">
         <is>
-          <t>NOT NULL</t>
+          <t>NOT NULL DEFAULT TRUE</t>
         </is>
       </c>
       <c r="F17" s="9" t="inlineStr">
         <is>
-          <t>Doctor degree &amp; credentials (e.g. MBBS, MD, DM)</t>
+          <t>Doctor active practicing availability flag</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="10" t="inlineStr">
         <is>
-          <t>doctors</t>
+          <t>doctor_availability</t>
         </is>
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>experience_years</t>
+          <t>id</t>
         </is>
       </c>
       <c r="C18" s="9" t="inlineStr">
         <is>
-          <t>INT</t>
+          <t>BIGINT AUTO_INCREMENT</t>
         </is>
       </c>
       <c r="D18" s="15" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>PRIMARY KEY</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
         <is>
-          <t>DEFAULT 0</t>
+          <t>NOT NULL</t>
         </is>
       </c>
       <c r="F18" s="9" t="inlineStr">
         <is>
-          <t>Years of clinical practicing experience</t>
+          <t>Unique availability schedule primary key identifier</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="10" t="inlineStr">
         <is>
-          <t>doctors</t>
+          <t>doctor_availability</t>
         </is>
       </c>
       <c r="B19" s="10" t="inlineStr">
         <is>
-          <t>consultation_fee</t>
+          <t>doctor_id</t>
         </is>
       </c>
       <c r="C19" s="9" t="inlineStr">
         <is>
-          <t>DECIMAL(10,2)</t>
+          <t>BIGINT</t>
         </is>
       </c>
       <c r="D19" s="15" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>FOREIGN KEY</t>
         </is>
       </c>
       <c r="E19" s="9" t="inlineStr">
@@ -2708,24 +2765,24 @@
       </c>
       <c r="F19" s="9" t="inlineStr">
         <is>
-          <t>Doctor outpatient consultation fee</t>
+          <t>Many:1 reference to doctors(id) ON DELETE CASCADE</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="10" t="inlineStr">
         <is>
-          <t>doctors</t>
+          <t>doctor_availability</t>
         </is>
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>is_active</t>
+          <t>day_of_week</t>
         </is>
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>BOOLEAN</t>
+          <t>ENUM('MONDAY'..'SUNDAY')</t>
         </is>
       </c>
       <c r="D20" s="15" t="inlineStr">
@@ -2735,34 +2792,34 @@
       </c>
       <c r="E20" s="9" t="inlineStr">
         <is>
-          <t>DEFAULT TRUE</t>
+          <t>NOT NULL</t>
         </is>
       </c>
       <c r="F20" s="9" t="inlineStr">
         <is>
-          <t>Doctor active practicing status flag</t>
+          <t>Working day of week enum for scheduled clinical shifts</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="10" t="inlineStr">
         <is>
-          <t>doctor_availabilities</t>
+          <t>doctor_availability</t>
         </is>
       </c>
       <c r="B21" s="10" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>start_time</t>
         </is>
       </c>
       <c r="C21" s="9" t="inlineStr">
         <is>
-          <t>BIGINT AUTO_INCREMENT</t>
+          <t>TIME</t>
         </is>
       </c>
       <c r="D21" s="15" t="inlineStr">
         <is>
-          <t>PRIMARY KEY</t>
+          <t>NONE</t>
         </is>
       </c>
       <c r="E21" s="9" t="inlineStr">
@@ -2772,29 +2829,29 @@
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
-          <t>Unique availability schedule primary key</t>
+          <t>Shift consultation start time (e.g. 09:00:00)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="10" t="inlineStr">
         <is>
-          <t>doctor_availabilities</t>
+          <t>doctor_availability</t>
         </is>
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>doctor_id</t>
+          <t>end_time</t>
         </is>
       </c>
       <c r="C22" s="9" t="inlineStr">
         <is>
-          <t>BIGINT</t>
+          <t>TIME</t>
         </is>
       </c>
       <c r="D22" s="15" t="inlineStr">
         <is>
-          <t>FOREIGN KEY</t>
+          <t>NONE</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -2804,61 +2861,61 @@
       </c>
       <c r="F22" s="9" t="inlineStr">
         <is>
-          <t>References doctors(id) ON DELETE CASCADE</t>
+          <t>Shift consultation end time (e.g. 13:00:00)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="10" t="inlineStr">
         <is>
-          <t>doctor_availabilities</t>
+          <t>doctor_availability</t>
         </is>
       </c>
       <c r="B23" s="10" t="inlineStr">
         <is>
-          <t>day_of_week</t>
+          <t>uk_doc_day</t>
         </is>
       </c>
       <c r="C23" s="9" t="inlineStr">
         <is>
-          <t>VARCHAR(20)</t>
+          <t>UNIQUE KEY</t>
         </is>
       </c>
       <c r="D23" s="15" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>COMPOSITE UNIQUE</t>
         </is>
       </c>
       <c r="E23" s="9" t="inlineStr">
         <is>
-          <t>NOT NULL</t>
+          <t>CONSTRAINT</t>
         </is>
       </c>
       <c r="F23" s="9" t="inlineStr">
         <is>
-          <t>Day of week (MONDAY, TUESDAY, ..., SATURDAY)</t>
+          <t>Unique constraint on (doctor_id, day_of_week) preventing overlapping shifts</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="10" t="inlineStr">
         <is>
-          <t>doctor_availabilities</t>
+          <t>patients</t>
         </is>
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>start_time</t>
+          <t>id</t>
         </is>
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t>TIME</t>
+          <t>BIGINT AUTO_INCREMENT</t>
         </is>
       </c>
       <c r="D24" s="15" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>PRIMARY KEY</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -2868,29 +2925,29 @@
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
-          <t>Shift consultation start time (e.g. 09:00:00)</t>
+          <t>Unique patient medical profile primary key identifier</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="10" t="inlineStr">
         <is>
-          <t>doctor_availabilities</t>
+          <t>patients</t>
         </is>
       </c>
       <c r="B25" s="10" t="inlineStr">
         <is>
-          <t>end_time</t>
+          <t>user_id</t>
         </is>
       </c>
       <c r="C25" s="9" t="inlineStr">
         <is>
-          <t>TIME</t>
+          <t>BIGINT</t>
         </is>
       </c>
       <c r="D25" s="15" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>FOREIGN KEY &amp; UNIQUE</t>
         </is>
       </c>
       <c r="E25" s="9" t="inlineStr">
@@ -2900,24 +2957,24 @@
       </c>
       <c r="F25" s="9" t="inlineStr">
         <is>
-          <t>Shift consultation end time (e.g. 13:00:00)</t>
+          <t>1:1 reference to users(id) ON DELETE CASCADE</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="10" t="inlineStr">
         <is>
-          <t>doctor_availabilities</t>
+          <t>patients</t>
         </is>
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>slot_duration_minutes</t>
+          <t>phone</t>
         </is>
       </c>
       <c r="C26" s="9" t="inlineStr">
         <is>
-          <t>INT</t>
+          <t>VARCHAR(20)</t>
         </is>
       </c>
       <c r="D26" s="15" t="inlineStr">
@@ -2927,12 +2984,12 @@
       </c>
       <c r="E26" s="9" t="inlineStr">
         <is>
-          <t>DEFAULT 30</t>
+          <t>NOT NULL</t>
         </is>
       </c>
       <c r="F26" s="9" t="inlineStr">
         <is>
-          <t>Consultation slot interval duration (30 mins)</t>
+          <t>Patient primary contact telephone number</t>
         </is>
       </c>
     </row>
@@ -2944,27 +3001,27 @@
       </c>
       <c r="B27" s="10" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>dob</t>
         </is>
       </c>
       <c r="C27" s="9" t="inlineStr">
         <is>
-          <t>BIGINT AUTO_INCREMENT</t>
+          <t>DATE</t>
         </is>
       </c>
       <c r="D27" s="15" t="inlineStr">
         <is>
-          <t>PRIMARY KEY</t>
+          <t>NONE</t>
         </is>
       </c>
       <c r="E27" s="9" t="inlineStr">
         <is>
-          <t>NOT NULL</t>
+          <t>NULL</t>
         </is>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>Unique patient primary key identifier</t>
+          <t>Patient date of birth for age calculation and clinical records</t>
         </is>
       </c>
     </row>
@@ -2976,27 +3033,27 @@
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>user_id</t>
+          <t>gender</t>
         </is>
       </c>
       <c r="C28" s="9" t="inlineStr">
         <is>
-          <t>BIGINT</t>
+          <t>VARCHAR(10)</t>
         </is>
       </c>
       <c r="D28" s="15" t="inlineStr">
         <is>
-          <t>FOREIGN KEY</t>
+          <t>NONE</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
         <is>
-          <t>NOT NULL</t>
+          <t>NULL</t>
         </is>
       </c>
       <c r="F28" s="9" t="inlineStr">
         <is>
-          <t>References users(id) ON DELETE CASCADE</t>
+          <t>Patient gender identifier (MALE, FEMALE, OTHER)</t>
         </is>
       </c>
     </row>
@@ -3008,12 +3065,12 @@
       </c>
       <c r="B29" s="10" t="inlineStr">
         <is>
-          <t>date_of_birth</t>
+          <t>address</t>
         </is>
       </c>
       <c r="C29" s="9" t="inlineStr">
         <is>
-          <t>DATE</t>
+          <t>VARCHAR(255)</t>
         </is>
       </c>
       <c r="D29" s="15" t="inlineStr">
@@ -3028,103 +3085,103 @@
       </c>
       <c r="F29" s="9" t="inlineStr">
         <is>
-          <t>Patient birth date for age computation</t>
+          <t>Patient residential postal address</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="10" t="inlineStr">
         <is>
-          <t>patients</t>
+          <t>appointments</t>
         </is>
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>gender</t>
+          <t>id</t>
         </is>
       </c>
       <c r="C30" s="9" t="inlineStr">
         <is>
-          <t>VARCHAR(10)</t>
+          <t>BIGINT AUTO_INCREMENT</t>
         </is>
       </c>
       <c r="D30" s="15" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>PRIMARY KEY</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>NOT NULL</t>
         </is>
       </c>
       <c r="F30" s="9" t="inlineStr">
         <is>
-          <t>Patient gender (MALE, FEMALE, OTHER)</t>
+          <t>Unique appointment booking record primary key identifier</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="10" t="inlineStr">
         <is>
-          <t>patients</t>
+          <t>appointments</t>
         </is>
       </c>
       <c r="B31" s="10" t="inlineStr">
         <is>
-          <t>blood_group</t>
+          <t>patient_id</t>
         </is>
       </c>
       <c r="C31" s="9" t="inlineStr">
         <is>
-          <t>VARCHAR(10)</t>
+          <t>BIGINT</t>
         </is>
       </c>
       <c r="D31" s="15" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>FOREIGN KEY</t>
         </is>
       </c>
       <c r="E31" s="9" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>NOT NULL</t>
         </is>
       </c>
       <c r="F31" s="9" t="inlineStr">
         <is>
-          <t>Patient blood group (A+, B+, O+, AB+, etc.)</t>
+          <t>Many:1 reference to patients(id)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="10" t="inlineStr">
         <is>
-          <t>patients</t>
+          <t>appointments</t>
         </is>
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>address</t>
+          <t>doctor_id</t>
         </is>
       </c>
       <c r="C32" s="9" t="inlineStr">
         <is>
-          <t>TEXT</t>
+          <t>BIGINT</t>
         </is>
       </c>
       <c r="D32" s="15" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>FOREIGN KEY</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>NOT NULL</t>
         </is>
       </c>
       <c r="F32" s="9" t="inlineStr">
         <is>
-          <t>Patient residential address</t>
+          <t>Many:1 reference to doctors(id)</t>
         </is>
       </c>
     </row>
@@ -3136,17 +3193,17 @@
       </c>
       <c r="B33" s="10" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>appointment_date</t>
         </is>
       </c>
       <c r="C33" s="9" t="inlineStr">
         <is>
-          <t>BIGINT AUTO_INCREMENT</t>
+          <t>DATE</t>
         </is>
       </c>
       <c r="D33" s="15" t="inlineStr">
         <is>
-          <t>PRIMARY KEY</t>
+          <t>NONE</t>
         </is>
       </c>
       <c r="E33" s="9" t="inlineStr">
@@ -3156,7 +3213,7 @@
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
-          <t>Unique appointment primary key identifier</t>
+          <t>Calendar date of scheduled medical consultation</t>
         </is>
       </c>
     </row>
@@ -3168,17 +3225,17 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>patient_id</t>
+          <t>appointment_time</t>
         </is>
       </c>
       <c r="C34" s="9" t="inlineStr">
         <is>
-          <t>BIGINT</t>
+          <t>TIME</t>
         </is>
       </c>
       <c r="D34" s="15" t="inlineStr">
         <is>
-          <t>FOREIGN KEY</t>
+          <t>NONE</t>
         </is>
       </c>
       <c r="E34" s="9" t="inlineStr">
@@ -3188,7 +3245,7 @@
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
-          <t>References patients(id)</t>
+          <t>Booked 30-minute consultation time slot (e.g. 10:00:00)</t>
         </is>
       </c>
     </row>
@@ -3200,17 +3257,17 @@
       </c>
       <c r="B35" s="10" t="inlineStr">
         <is>
-          <t>doctor_id</t>
+          <t>token_number</t>
         </is>
       </c>
       <c r="C35" s="9" t="inlineStr">
         <is>
-          <t>BIGINT</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D35" s="15" t="inlineStr">
         <is>
-          <t>FOREIGN KEY</t>
+          <t>NONE</t>
         </is>
       </c>
       <c r="E35" s="9" t="inlineStr">
@@ -3220,7 +3277,7 @@
       </c>
       <c r="F35" s="9" t="inlineStr">
         <is>
-          <t>References doctors(id)</t>
+          <t>Sequential daily queue token number per doctor per date (1, 2, 3...)</t>
         </is>
       </c>
     </row>
@@ -3232,12 +3289,12 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>appointment_date</t>
+          <t>status</t>
         </is>
       </c>
       <c r="C36" s="9" t="inlineStr">
         <is>
-          <t>DATE</t>
+          <t>ENUM('BOOKED','IN_CONSULTATION','COMPLETED','CANCELLED')</t>
         </is>
       </c>
       <c r="D36" s="15" t="inlineStr">
@@ -3247,12 +3304,12 @@
       </c>
       <c r="E36" s="9" t="inlineStr">
         <is>
-          <t>NOT NULL</t>
+          <t>DEFAULT 'BOOKED'</t>
         </is>
       </c>
       <c r="F36" s="9" t="inlineStr">
         <is>
-          <t>Date of scheduled consultation</t>
+          <t>Consultation workflow lifecycle state enum</t>
         </is>
       </c>
     </row>
@@ -3264,12 +3321,12 @@
       </c>
       <c r="B37" s="10" t="inlineStr">
         <is>
-          <t>slot_time</t>
+          <t>created_at</t>
         </is>
       </c>
       <c r="C37" s="9" t="inlineStr">
         <is>
-          <t>TIME</t>
+          <t>TIMESTAMP</t>
         </is>
       </c>
       <c r="D37" s="15" t="inlineStr">
@@ -3279,12 +3336,12 @@
       </c>
       <c r="E37" s="9" t="inlineStr">
         <is>
-          <t>NOT NULL</t>
+          <t>DEFAULT CURRENT_TIMESTAMP</t>
         </is>
       </c>
       <c r="F37" s="9" t="inlineStr">
         <is>
-          <t>Booked 30-min time slot (e.g. 10:00:00)</t>
+          <t>Appointment booking creation timestamp</t>
         </is>
       </c>
     </row>
@@ -3296,49 +3353,49 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>uk_doctor_slot</t>
         </is>
       </c>
       <c r="C38" s="9" t="inlineStr">
         <is>
-          <t>VARCHAR(20)</t>
+          <t>UNIQUE KEY</t>
         </is>
       </c>
       <c r="D38" s="15" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>COMPOSITE UNIQUE</t>
         </is>
       </c>
       <c r="E38" s="9" t="inlineStr">
         <is>
-          <t>DEFAULT "PENDING"</t>
+          <t>CONSTRAINT</t>
         </is>
       </c>
       <c r="F38" s="9" t="inlineStr">
         <is>
-          <t>Status: PENDING, CONFIRMED, IN_CONSULTATION, COMPLETED, CANCELLED</t>
+          <t>Strict unique constraint on (doctor_id, appointment_date, appointment_time) preventing double-booking</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="10" t="inlineStr">
         <is>
-          <t>appointments</t>
+          <t>prescriptions</t>
         </is>
       </c>
       <c r="B39" s="10" t="inlineStr">
         <is>
-          <t>token_number</t>
+          <t>id</t>
         </is>
       </c>
       <c r="C39" s="9" t="inlineStr">
         <is>
-          <t>INT</t>
+          <t>BIGINT AUTO_INCREMENT</t>
         </is>
       </c>
       <c r="D39" s="15" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>PRIMARY KEY</t>
         </is>
       </c>
       <c r="E39" s="9" t="inlineStr">
@@ -3348,56 +3405,56 @@
       </c>
       <c r="F39" s="9" t="inlineStr">
         <is>
-          <t>Sequential token number per doctor per date</t>
+          <t>Unique clinical prescription document primary key identifier</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="10" t="inlineStr">
         <is>
-          <t>appointments</t>
+          <t>prescriptions</t>
         </is>
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>reason_for_visit</t>
+          <t>appointment_id</t>
         </is>
       </c>
       <c r="C40" s="9" t="inlineStr">
         <is>
-          <t>TEXT</t>
+          <t>BIGINT</t>
         </is>
       </c>
       <c r="D40" s="15" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>FOREIGN KEY &amp; UNIQUE</t>
         </is>
       </c>
       <c r="E40" s="9" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>NOT NULL</t>
         </is>
       </c>
       <c r="F40" s="9" t="inlineStr">
         <is>
-          <t>Chief medical complaint or visit reason</t>
+          <t>1:1 reference to appointments(id) ON DELETE CASCADE</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="10" t="inlineStr">
         <is>
-          <t>appointments</t>
+          <t>prescriptions</t>
         </is>
       </c>
       <c r="B41" s="10" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>diagnosis</t>
         </is>
       </c>
       <c r="C41" s="9" t="inlineStr">
         <is>
-          <t>TIMESTAMP</t>
+          <t>TEXT</t>
         </is>
       </c>
       <c r="D41" s="15" t="inlineStr">
@@ -3407,29 +3464,29 @@
       </c>
       <c r="E41" s="9" t="inlineStr">
         <is>
-          <t>DEFAULT CURRENT_TIMESTAMP</t>
+          <t>NOT NULL</t>
         </is>
       </c>
       <c r="F41" s="9" t="inlineStr">
         <is>
-          <t>Booking creation timestamp</t>
+          <t>Doctor diagnostic assessment and clinical observations</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="10" t="inlineStr">
         <is>
-          <t>appointments</t>
+          <t>prescriptions</t>
         </is>
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>updated_at</t>
+          <t>notes</t>
         </is>
       </c>
       <c r="C42" s="9" t="inlineStr">
         <is>
-          <t>TIMESTAMP</t>
+          <t>TEXT</t>
         </is>
       </c>
       <c r="D42" s="15" t="inlineStr">
@@ -3439,12 +3496,12 @@
       </c>
       <c r="E42" s="9" t="inlineStr">
         <is>
-          <t>DEFAULT CURRENT_TIMESTAMP ON UPDATE</t>
+          <t>NULL</t>
         </is>
       </c>
       <c r="F42" s="9" t="inlineStr">
         <is>
-          <t>Last modification audit timestamp</t>
+          <t>Clinical advice, dietary precautions, and follow-up guidance</t>
         </is>
       </c>
     </row>
@@ -3456,49 +3513,49 @@
       </c>
       <c r="B43" s="10" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>created_at</t>
         </is>
       </c>
       <c r="C43" s="9" t="inlineStr">
         <is>
-          <t>BIGINT AUTO_INCREMENT</t>
+          <t>TIMESTAMP</t>
         </is>
       </c>
       <c r="D43" s="15" t="inlineStr">
         <is>
-          <t>PRIMARY KEY</t>
+          <t>NONE</t>
         </is>
       </c>
       <c r="E43" s="9" t="inlineStr">
         <is>
-          <t>NOT NULL</t>
+          <t>DEFAULT CURRENT_TIMESTAMP</t>
         </is>
       </c>
       <c r="F43" s="9" t="inlineStr">
         <is>
-          <t>Unique prescription primary key identifier</t>
+          <t>Prescription generation timestamp</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t>prescriptions</t>
+          <t>prescription_medicines</t>
         </is>
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>appointment_id</t>
+          <t>id</t>
         </is>
       </c>
       <c r="C44" s="9" t="inlineStr">
         <is>
-          <t>BIGINT</t>
+          <t>BIGINT AUTO_INCREMENT</t>
         </is>
       </c>
       <c r="D44" s="15" t="inlineStr">
         <is>
-          <t>FOREIGN KEY (UNIQUE)</t>
+          <t>PRIMARY KEY</t>
         </is>
       </c>
       <c r="E44" s="9" t="inlineStr">
@@ -3508,29 +3565,29 @@
       </c>
       <c r="F44" s="9" t="inlineStr">
         <is>
-          <t>References appointments(id) (1:1 relationship)</t>
+          <t>Unique prescribed medication item primary key identifier</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="10" t="inlineStr">
         <is>
-          <t>prescriptions</t>
+          <t>prescription_medicines</t>
         </is>
       </c>
       <c r="B45" s="10" t="inlineStr">
         <is>
-          <t>diagnosis</t>
+          <t>prescription_id</t>
         </is>
       </c>
       <c r="C45" s="9" t="inlineStr">
         <is>
-          <t>TEXT</t>
+          <t>BIGINT</t>
         </is>
       </c>
       <c r="D45" s="15" t="inlineStr">
         <is>
-          <t>NONE</t>
+          <t>FOREIGN KEY</t>
         </is>
       </c>
       <c r="E45" s="9" t="inlineStr">
@@ -3540,24 +3597,24 @@
       </c>
       <c r="F45" s="9" t="inlineStr">
         <is>
-          <t>Doctor clinical diagnosis text</t>
+          <t>Many:1 reference to prescriptions(id) ON DELETE CASCADE</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="10" t="inlineStr">
         <is>
-          <t>prescriptions</t>
+          <t>prescription_medicines</t>
         </is>
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>clinical_notes</t>
+          <t>medicine_name</t>
         </is>
       </c>
       <c r="C46" s="9" t="inlineStr">
         <is>
-          <t>TEXT</t>
+          <t>VARCHAR(150)</t>
         </is>
       </c>
       <c r="D46" s="15" t="inlineStr">
@@ -3567,29 +3624,29 @@
       </c>
       <c r="E46" s="9" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>NOT NULL</t>
         </is>
       </c>
       <c r="F46" s="9" t="inlineStr">
         <is>
-          <t>Advice, dietary guidance, and doctor notes</t>
+          <t>Pharmaceutical brand or generic medicine name (e.g. Paracetamol, Amlodipine)</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="10" t="inlineStr">
         <is>
-          <t>prescriptions</t>
+          <t>prescription_medicines</t>
         </is>
       </c>
       <c r="B47" s="10" t="inlineStr">
         <is>
-          <t>follow_up_date</t>
+          <t>dosage</t>
         </is>
       </c>
       <c r="C47" s="9" t="inlineStr">
         <is>
-          <t>DATE</t>
+          <t>VARCHAR(50)</t>
         </is>
       </c>
       <c r="D47" s="15" t="inlineStr">
@@ -3599,29 +3656,29 @@
       </c>
       <c r="E47" s="9" t="inlineStr">
         <is>
-          <t>NULL</t>
+          <t>NOT NULL</t>
         </is>
       </c>
       <c r="F47" s="9" t="inlineStr">
         <is>
-          <t>Recommended follow-up visit date</t>
+          <t>Medication dosage quantity/strength (e.g. 500mg, 1 tablet, 5ml)</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="10" t="inlineStr">
         <is>
-          <t>prescriptions</t>
+          <t>prescription_medicines</t>
         </is>
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>frequency</t>
         </is>
       </c>
       <c r="C48" s="9" t="inlineStr">
         <is>
-          <t>TIMESTAMP</t>
+          <t>VARCHAR(50)</t>
         </is>
       </c>
       <c r="D48" s="15" t="inlineStr">
@@ -3631,12 +3688,12 @@
       </c>
       <c r="E48" s="9" t="inlineStr">
         <is>
-          <t>DEFAULT CURRENT_TIMESTAMP</t>
+          <t>NOT NULL</t>
         </is>
       </c>
       <c r="F48" s="9" t="inlineStr">
         <is>
-          <t>Prescription generation timestamp</t>
+          <t>Dosage schedule frequency (e.g. 1-0-1, 1-1-1, 0-0-1 after meals)</t>
         </is>
       </c>
     </row>
@@ -3648,17 +3705,17 @@
       </c>
       <c r="B49" s="10" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>duration</t>
         </is>
       </c>
       <c r="C49" s="9" t="inlineStr">
         <is>
-          <t>BIGINT AUTO_INCREMENT</t>
+          <t>VARCHAR(50)</t>
         </is>
       </c>
       <c r="D49" s="15" t="inlineStr">
         <is>
-          <t>PRIMARY KEY</t>
+          <t>NONE</t>
         </is>
       </c>
       <c r="E49" s="9" t="inlineStr">
@@ -3668,7 +3725,7 @@
       </c>
       <c r="F49" s="9" t="inlineStr">
         <is>
-          <t>Unique prescribed medicine item identifier</t>
+          <t>Course duration length (e.g. 5 days, 10 days, 1 month)</t>
         </is>
       </c>
     </row>
@@ -3680,27 +3737,27 @@
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>prescription_id</t>
+          <t>instructions</t>
         </is>
       </c>
       <c r="C50" s="9" t="inlineStr">
         <is>
-          <t>BIGINT</t>
+          <t>VARCHAR(255)</t>
         </is>
       </c>
       <c r="D50" s="15" t="inlineStr">
         <is>
-          <t>FOREIGN KEY</t>
+          <t>NONE</t>
         </is>
       </c>
       <c r="E50" s="9" t="inlineStr">
         <is>
-          <t>NOT NULL</t>
+          <t>NULL</t>
         </is>
       </c>
       <c r="F50" s="9" t="inlineStr">
         <is>
-          <t>References prescriptions(id) ON DELETE CASCADE</t>
+          <t>Specific administration instructions (e.g. Take with warm water after food)</t>
         </is>
       </c>
     </row>
@@ -3875,7 +3932,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -3890,11 +3947,10 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>🌐 PHASE 2: DESIGN — RESTFUL API CONTRACTS &amp; POSTMAN SPECS</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
+          <t>🌐 PHASE 2: DESIGN — RESTFUL API SPECIFICATIONS &amp; POSTMAN CONTRACTS</t>
+        </is>
+      </c>
+    </row>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
         <is>
@@ -3945,10 +4001,59 @@
       </c>
       <c r="C4" s="9" t="inlineStr">
         <is>
+          <t>/api/auth/register</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>{
+  "name": "Jane Doe",
+  "email": "jane@clinic.com",
+  "password": "password123",
+  "role": "PATIENT",
+  "phone": "9876543210"
+}</t>
+        </is>
+      </c>
+      <c r="E4" s="15" t="inlineStr">
+        <is>
+          <t>201 Created</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>{
+  "id": 5,
+  "name": "Jane Doe",
+  "email": "jane@clinic.com",
+  "role": "PATIENT",
+  "message": "User registered successfully"
+}</t>
+        </is>
+      </c>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>400 Bad Request (Email already registered / validation error)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="55" customHeight="1">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>API-02</t>
+        </is>
+      </c>
+      <c r="B5" s="15" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
           <t>/api/auth/login</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="D5" s="9" t="inlineStr">
         <is>
           <t>{
   "email": "patient@clinic.com",
@@ -3956,12 +4061,12 @@
 }</t>
         </is>
       </c>
-      <c r="E4" s="15" t="inlineStr">
+      <c r="E5" s="15" t="inlineStr">
         <is>
           <t>200 OK</t>
         </is>
       </c>
-      <c r="F4" s="9" t="inlineStr">
+      <c r="F5" s="9" t="inlineStr">
         <is>
           <t>{
   "id": 1,
@@ -3972,39 +4077,84 @@
 }</t>
         </is>
       </c>
-      <c r="G4" s="9" t="inlineStr">
-        <is>
-          <t>400 Bad Request / 401 Unauthorized (Invalid email/password)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="55" customHeight="1">
-      <c r="A5" s="10" t="inlineStr">
-        <is>
-          <t>API-02</t>
-        </is>
-      </c>
-      <c r="B5" s="15" t="inlineStr">
+      <c r="G5" s="9" t="inlineStr">
+        <is>
+          <t>400 Bad Request / 401 Unauthorized (Invalid email or password)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="55" customHeight="1">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>API-03</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="C5" s="9" t="inlineStr">
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>/api/doctors</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>None (Empty Body)</t>
+        </is>
+      </c>
+      <c r="E6" s="15" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>[
+  {
+    "id": 1,
+    "name": "Dr. Ramesh Kumar",
+    "specializationName": "Cardiology",
+    "consultationFee": 500.00,
+    "available": true
+  }
+]</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>500 Internal Server Error</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="55" customHeight="1">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>API-04</t>
+        </is>
+      </c>
+      <c r="B7" s="15" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
         <is>
           <t>/api/doctors/{id}/slots?date=2026-09-20</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="D7" s="9" t="inlineStr">
         <is>
           <t>None (Query Param: date)</t>
         </is>
       </c>
-      <c r="E5" s="15" t="inlineStr">
+      <c r="E7" s="15" t="inlineStr">
         <is>
           <t>200 OK</t>
         </is>
       </c>
-      <c r="F5" s="9" t="inlineStr">
+      <c r="F7" s="9" t="inlineStr">
         <is>
           <t>{
   "doctorId": 1,
@@ -4017,29 +4167,29 @@
 }</t>
         </is>
       </c>
-      <c r="G5" s="9" t="inlineStr">
+      <c r="G7" s="9" t="inlineStr">
         <is>
           <t>404 Not Found (Doctor not found or no schedule on this day)</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="55" customHeight="1">
-      <c r="A6" s="10" t="inlineStr">
-        <is>
-          <t>API-03</t>
-        </is>
-      </c>
-      <c r="B6" s="15" t="inlineStr">
+    <row r="8" ht="55" customHeight="1">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>API-05</t>
+        </is>
+      </c>
+      <c r="B8" s="15" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>/api/appointments</t>
         </is>
       </c>
-      <c r="D6" s="9" t="inlineStr">
+      <c r="D8" s="9" t="inlineStr">
         <is>
           <t>{
   "doctorId": 1,
@@ -4049,12 +4199,12 @@
 }</t>
         </is>
       </c>
-      <c r="E6" s="15" t="inlineStr">
+      <c r="E8" s="15" t="inlineStr">
         <is>
           <t>201 Created</t>
         </is>
       </c>
-      <c r="F6" s="9" t="inlineStr">
+      <c r="F8" s="9" t="inlineStr">
         <is>
           <t>{
   "id": 101,
@@ -4066,78 +4216,123 @@
 }</t>
         </is>
       </c>
-      <c r="G6" s="9" t="inlineStr">
+      <c r="G8" s="9" t="inlineStr">
         <is>
           <t>400 Bad Request (Missing fields) / 409 Conflict (Slot already booked)</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="55" customHeight="1">
-      <c r="A7" s="10" t="inlineStr">
-        <is>
-          <t>API-04</t>
-        </is>
-      </c>
-      <c r="B7" s="15" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>API-06</t>
+        </is>
+      </c>
+      <c r="B9" s="15" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>/api/appointments/patient/{patientId}</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>None (Patient ID in Path)</t>
+        </is>
+      </c>
+      <c r="E9" s="15" t="inlineStr">
+        <is>
+          <t>200 OK</t>
+        </is>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>[
+  {
+    "id": 101,
+    "doctorName": "Dr. Ramesh Kumar",
+    "appointmentDate": "2026-09-20",
+    "slotTime": "09:00",
+    "tokenNumber": 1,
+    "status": "CONFIRMED"
+  }
+]</t>
+        </is>
+      </c>
+      <c r="G9" s="9" t="inlineStr">
+        <is>
+          <t>404 Not Found (Patient not found)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>API-07</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="inlineStr">
         <is>
           <t>PUT</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr">
+      <c r="C10" s="9" t="inlineStr">
         <is>
           <t>/api/appointments/{id}/status</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="D10" s="9" t="inlineStr">
         <is>
           <t>{
   "status": "IN_CONSULTATION"
 }</t>
         </is>
       </c>
-      <c r="E7" s="15" t="inlineStr">
+      <c r="E10" s="15" t="inlineStr">
         <is>
           <t>200 OK</t>
         </is>
       </c>
-      <c r="F7" s="9" t="inlineStr">
+      <c r="F10" s="9" t="inlineStr">
         <is>
           <t>{
   "id": 101,
   "status": "IN_CONSULTATION",
-  "updatedAt": "2026-09-18T10:30:00Z"
+  "updatedAt": "2026-09-19T10:30:00Z"
 }</t>
         </is>
       </c>
-      <c r="G7" s="9" t="inlineStr">
+      <c r="G10" s="9" t="inlineStr">
         <is>
           <t>404 Not Found / 400 Bad Request (Invalid status transition)</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="55" customHeight="1">
-      <c r="A8" s="10" t="inlineStr">
-        <is>
-          <t>API-05</t>
-        </is>
-      </c>
-      <c r="B8" s="15" t="inlineStr">
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>API-08</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>/api/prescriptions</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>{
   "appointmentId": 101,
   "diagnosis": "Mild Hypertension",
-  "clinicalNotes": "Maintain low-sodium diet",
-  "followUpDate": "2026-10-05",
+  "notes": "Maintain low-sodium diet and exercise",
   "medicines": [
     {
       "medicineName": "Amlodipine 5mg",
@@ -4150,12 +4345,12 @@
 }</t>
         </is>
       </c>
-      <c r="E8" s="15" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>201 Created</t>
         </is>
       </c>
-      <c r="F8" s="9" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>{
   "id": 51,
@@ -4165,45 +4360,47 @@
     {
       "id": 81,
       "medicineName": "Amlodipine 5mg",
-      "dosage": "1 tablet"
+      "dosage": "1 tablet",
+      "frequency": "0-0-1",
+      "duration": "15 days"
     }
   ]
 }</t>
         </is>
       </c>
-      <c r="G8" s="9" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>400 Bad Request / 404 Not Found (Appointment does not exist)</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="10" t="inlineStr">
-        <is>
-          <t>API-06</t>
-        </is>
-      </c>
-      <c r="B9" s="15" t="inlineStr">
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>API-09</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>/api/queue/doctor/{doctorId}/today</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>None (Doctor ID in Path)</t>
         </is>
       </c>
-      <c r="E9" s="15" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>200 OK</t>
         </is>
       </c>
-      <c r="F9" s="9" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>{
   "doctorId": 1,
@@ -4222,39 +4419,39 @@
 }</t>
         </is>
       </c>
-      <c r="G9" s="9" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>404 Not Found (Doctor does not exist)</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="10" t="inlineStr">
-        <is>
-          <t>API-07</t>
-        </is>
-      </c>
-      <c r="B10" s="15" t="inlineStr">
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>API-10</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>/api/admin/stats</t>
         </is>
       </c>
-      <c r="D10" s="9" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>None (Empty Body)</t>
         </is>
       </c>
-      <c r="E10" s="15" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>200 OK</t>
         </is>
       </c>
-      <c r="F10" s="9" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>{
   "totalDoctors": 6,
@@ -4264,7 +4461,7 @@
 }</t>
         </is>
       </c>
-      <c r="G10" s="9" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>500 Internal Server Error</t>
         </is>
@@ -4295,11 +4492,10 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>🤖 PHASE 3: DEVELOP — CARE AI PROMPT ENGINEERING LOG</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
+          <t>🤖 PHASE 3: DEVELOP — CARE AI PROMPT ENGINEERING &amp; AUDIT LOG</t>
+        </is>
+      </c>
+    </row>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
         <is>
@@ -4340,12 +4536,12 @@
       </c>
       <c r="B4" s="16" t="inlineStr">
         <is>
-          <t>Anti Gravity / Claude</t>
+          <t>Antigravity IDE / Gemini 3.7</t>
         </is>
       </c>
       <c r="C4" s="9" t="inlineStr">
         <is>
-          <t>Generate Spring Boot JPA Entities with Relationships</t>
+          <t>Generate Spring Boot JPA Entities with Bidirectional Relations &amp; JSON Controls</t>
         </is>
       </c>
       <c r="D4" s="9" t="inlineStr">
@@ -4358,12 +4554,12 @@
       </c>
       <c r="E4" s="9" t="inlineStr">
         <is>
-          <t>Generated Appointment.java and Prescription.java with @Entity, @Table(uniqueConstraints=...), and @OneToMany relations.</t>
+          <t>Generated User.java, Doctor.java, Appointment.java, Prescription.java with @Entity, @Table(uniqueConstraints=...), and @OneToMany relations.</t>
         </is>
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
-          <t>Verified entity relationships. Added @JsonIgnore on parent back-references to prevent infinite recursion during JSON serialization.</t>
+          <t>Verified entity relationships. Added @JsonIgnore on parent back-references and transitioned to DTOs to prevent Jackson circular reference infinite recursion.</t>
         </is>
       </c>
     </row>
@@ -4375,30 +4571,30 @@
       </c>
       <c r="B5" s="16" t="inlineStr">
         <is>
-          <t>Kiro / ChatGPT</t>
+          <t>Antigravity IDE / Gemini 3.7</t>
         </is>
       </c>
       <c r="C5" s="9" t="inlineStr">
         <is>
-          <t>Generate Dynamic 30-Min Slot Grid &amp; Live Queue UI</t>
+          <t>Generate Dynamic 30-Min Slot Grid &amp; Interactive Slot Picker UI</t>
         </is>
       </c>
       <c r="D5" s="9" t="inlineStr">
         <is>
-          <t>Context: Clinic patient booking portal.
-Action: Create CSS Grid component for doctor 30-minute consultation slots. Style available slots in subtle green with hover elevation, and disabled slots in muted gray.
-Result: Modern responsive CSS Grid.
+          <t>Context: Clinic patient appointment booking portal.
+Action: Create CSS Grid component for doctor 30-minute consultation slots. Style available slots in vibrant green with hover elevation, and booked/disabled slots in muted gray.
+Result: Modern responsive CSS Grid with dynamic state transitions.
 Example: Mobile viewport breakpoint at 768px.</t>
         </is>
       </c>
       <c r="E5" s="9" t="inlineStr">
         <is>
-          <t>Generated .slot-grid with repeat(auto-fit, minmax(90px, 1fr)) and state badges (.slot-available, .slot-booked).</t>
+          <t>Generated .slot-grid with repeat(auto-fit, minmax(90px, 1fr)) and state badges (.slot-available, .slot-booked) with interactive click event handlers.</t>
         </is>
       </c>
       <c r="F5" s="9" t="inlineStr">
         <is>
-          <t>Tested across mobile and desktop viewports. Slot cards dynamically toggle upon date selection change.</t>
+          <t>Tested across mobile (375px) and desktop (1920px) viewports. Slot buttons dynamically re-render upon date selection change via async Fetch API.</t>
         </is>
       </c>
     </row>
@@ -4410,7 +4606,7 @@
       </c>
       <c r="B6" s="16" t="inlineStr">
         <is>
-          <t>Anti Gravity</t>
+          <t>Antigravity IDE / Gemini 3.7</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
@@ -4423,17 +4619,17 @@
           <t>Context: Multi-user appointment booking API.
 Action: Design thread-safe booking logic in AppointmentService using database-level unique constraints and Spring Data JPA transaction isolation.
 Result: Service method + @ExceptionHandler.
-Example: SlotAlreadyBookedException returning 409 Conflict.</t>
+Example: SlotAlreadyBookedException returning HTTP 409 Conflict.</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
-          <t>Implemented existsByDoctorIdAndAppointmentDateAndSlotTimeAndStatusNot check + custom SlotAlreadyBookedException + GlobalExceptionHandler.</t>
+          <t>Implemented existsByDoctorIdAndAppointmentDateAndSlotTime check + custom SlotAlreadyBookedException + GlobalExceptionHandler (@RestControllerAdvice).</t>
         </is>
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t>Tested parallel curl requests targeting the same slot; 1st received 201 Created and 2nd was cleanly rejected with 409 Conflict.</t>
+          <t>Tested parallel curl/Postman requests targeting the same slot; 1st received 201 Created and 2nd was cleanly rejected with 409 Conflict.</t>
         </is>
       </c>
     </row>
@@ -4445,7 +4641,7 @@
       </c>
       <c r="B7" s="16" t="inlineStr">
         <is>
-          <t>Anti Gravity</t>
+          <t>Antigravity IDE / Gemini 3.7</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr">
@@ -4463,12 +4659,12 @@
       </c>
       <c r="E7" s="9" t="inlineStr">
         <is>
-          <t>Generated waiting-room.js with setInterval(fetchQueueStatus, 5000) and DOM diffing to prevent visual flicker.</t>
+          <t>Generated waiting-room.js with setInterval(fetchQueueStatus, 5000) and DOM diffing to prevent visual screen flicker.</t>
         </is>
       </c>
       <c r="F7" s="9" t="inlineStr">
         <is>
-          <t>Verified in browser. Display transitions automatically when doctor clicks "Call Next Patient" in another tab.</t>
+          <t>Verified in browser. Display transitions automatically within 5 seconds when doctor clicks 'Call Next Patient' in consultation console.</t>
         </is>
       </c>
     </row>
@@ -4496,11 +4692,10 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>🖥️ PHASE 3: DEVELOP — FRONTEND UI IMPLEMENTATION (HTML5 &amp; CSS3)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
+          <t>🖥️ PHASE 3: DEVELOP — FRONTEND UI IMPLEMENTATION (HTML5, CSS3 &amp; JS)</t>
+        </is>
+      </c>
+    </row>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
         <is>
@@ -4536,7 +4731,7 @@
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>&lt;header&gt;, &lt;nav&gt;, &lt;main&gt;, &lt;section&gt;, &lt;footer&gt;, CSS Variables, Flexbox Navbar</t>
+          <t>&lt;header&gt;, &lt;nav&gt;, &lt;main&gt;, &lt;section&gt;, &lt;footer&gt;, CSS Custom Properties, Flexbox Navbar</t>
         </is>
       </c>
       <c r="C4" s="9" t="inlineStr">
@@ -4546,7 +4741,7 @@
       </c>
       <c r="D4" s="9" t="inlineStr">
         <is>
-          <t>Implemented high-contrast modern clinic design system with CSS custom properties (--primary: #0284c7, --success: #16a34a), accessible typography, and mobile hamburger navigation.</t>
+          <t>Implemented modern medical design system with CSS tokens (--primary: #0284c7, --success: #16a34a), accessible typography, and mobile hamburger navigation.</t>
         </is>
       </c>
       <c r="E4" s="15" t="inlineStr">
@@ -4590,7 +4785,7 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>&lt;textarea&gt;, dynamic multi-row &lt;table id="medsTable"&gt;, "+ Add Medicine" button</t>
+          <t>&lt;textarea&gt;, dynamic multi-row &lt;table id="medsTable"&gt;, '+ Add Medicine' button</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
@@ -4627,7 +4822,7 @@
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
-          <t>Dedicated high-visibility display board optimized for clinic waiting room monitors showing "Current in Consultation", "Next in Line", and "Total Waiting" counters with smooth transitions.</t>
+          <t>Dedicated high-visibility display board optimized for clinic waiting room monitors showing 'Current in Consultation', 'Next in Line', and 'Total Waiting' counters with smooth transitions.</t>
         </is>
       </c>
       <c r="E7" s="15" t="inlineStr">
@@ -4687,11 +4882,10 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚙️ PHASE 3: DEVELOP — BACKEND &amp; MYSQL PERSISTENCE (SPRING BOOT)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
+          <t>⚙️ PHASE 3: DEVELOP — BACKEND ARCHITECTURE &amp; MYSQL PERSISTENCE (SPRING BOOT)</t>
+        </is>
+      </c>
+    </row>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
         <is>
@@ -4727,7 +4921,7 @@
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>application.properties, DataLoader.java</t>
+          <t>application.properties, DataLoader.java, SecurityConfig</t>
         </is>
       </c>
       <c r="C4" s="9" t="inlineStr">
@@ -4754,7 +4948,7 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>User.java, Doctor.java, Patient.java, Appointment.java, Prescription.java</t>
+          <t>User.java, Doctor.java, Patient.java, Appointment.java, Prescription.java, PrescriptionMedicine.java</t>
         </is>
       </c>
       <c r="C5" s="9" t="inlineStr">
@@ -4776,12 +4970,12 @@
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="15" t="inlineStr">
         <is>
-          <t>3. Data Repositories</t>
+          <t>3. Data Repositories (DAO)</t>
         </is>
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>AppointmentRepository.java, DoctorRepository.java, PrescriptionRepository.java</t>
+          <t>AppointmentRepository.java, DoctorRepository.java, PrescriptionRepository.java, UserRepository.java</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
@@ -4830,22 +5024,22 @@
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="15" t="inlineStr">
         <is>
-          <t>5. REST Controllers</t>
+          <t>5. REST Controllers &amp; Handlers</t>
         </is>
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>AppointmentController.java, DoctorController.java, QueueController.java, PrescriptionController.java</t>
+          <t>AppointmentController.java, DoctorController.java, QueueController.java, PrescriptionController.java, GlobalExceptionHandler.java</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>@RestController, @RequestMapping, @CrossOrigin, @PostMapping, @GetMapping</t>
+          <t>@RestController, @RequestMapping, @CrossOrigin, @PostMapping, @GetMapping, @RestControllerAdvice</t>
         </is>
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
-          <t>Exposed RESTful endpoints returning standardized JSON response envelopes, handling exceptions via @ControllerAdvice (GlobalExceptionHandler.java) with HTTP 200, 201, 400, 404, 409.</t>
+          <t>Exposed RESTful endpoints returning standardized JSON response envelopes, handling exceptions via @RestControllerAdvice with HTTP 200, 201, 400, 404, 409.</t>
         </is>
       </c>
       <c r="E8" s="15" t="inlineStr">

</xml_diff>